<commit_message>
SPM-94: Limit who sees a request's review outcome
Venue Staff, Technical Support and the Safety Officer see an event only
from Approved onwards; an unapproved request is the same 404 as a missing
one. The rejection reason goes only to the owning organiser, the assigned
coordinator and the Event Coordinator Lead (forum #125).

Also: fixtures (npm run fixtures:spm94), SPM-31-TC02 marked Updated, the
20261020 discussions export, and the #125 decision recorded in
CUSTOMER_CLARIFICATIONS.md.
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-31_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-31_Test_Cases.xlsx
@@ -698,11 +698,15 @@
       </c>
       <c r="G5" s="39" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H5" s="39" t="n"/>
-      <c r="I5" s="39" t="n"/>
+      <c r="I5" s="39" t="inlineStr">
+        <is>
+          <t>#125</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -18900,7 +18904,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="24.75" customWidth="1" style="35" min="1" max="1"/>
@@ -18909,235 +18913,241 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="35">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-23): Venue Staff, Technical Support and the Safety Officer now see an event only from Approved onwards (SPM-94 AC2, forum #125). Pearl Delta Safety Conference is in Planning, so the steps and result are unchanged; read 'internal staff can view any non-draft event' in the expected result as 'internal staff can view any event from Approved onwards (Event Coordinators and the Event Coordinator Lead: any non-draft event)'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17.25" customHeight="1" s="35">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" s="35">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="39" t="inlineStr">
-        <is>
-          <t>SPM-31-TC02</t>
-        </is>
-      </c>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3" ht="71.25" customHeight="1" s="35">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>SPM-31-TC02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30.75" customHeight="1" s="35">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="39" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Logged in as Marcus Wong (marcus.wong@connectsphere.com / password123), Venue Staff — not the coordinator, organiser, or attendee of any specific event.
 'Pearl Delta Safety Conference' (status Planning, coordinator Hui Shan Neo) exists.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30.75" customHeight="1" s="35">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="30.75" customHeight="1" s="35">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>1. Open 'All Events'
 2. Open 'Pearl Delta Safety Conference'</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30.75" customHeight="1" s="35">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="39" t="inlineStr">
-        <is>
-          <t>Event: Pearl Delta Safety Conference | Viewer role: Venue Staff</t>
-        </is>
-      </c>
-    </row>
     <row r="6" ht="44.25" customHeight="1" s="35">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Expected Result</t>
+          <t>Test Data</t>
         </is>
       </c>
       <c r="B6" s="39" t="inlineStr">
         <is>
-          <t>The event opens normally and its Overview details are shown — internal staff can view any non-draft event regardless of their own relationship to it.</t>
+          <t>Event: Pearl Delta Safety Conference | Viewer role: Venue Staff</t>
         </is>
       </c>
     </row>
     <row r="7" ht="17.25" customHeight="1" s="35">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Created By</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>The event opens normally and its Overview details are shown — internal staff can view any non-draft event regardless of their own relationship to it.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="35">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1" s="35">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B9" s="17" t="n">
         <v>46287</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="35"/>
-    <row r="10" ht="15.75" customHeight="1" s="35">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="35"/>
+    <row r="11" ht="15.75" customHeight="1" s="35">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="14" t="n"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1" s="35">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="39" t="inlineStr">
-        <is>
-          <t>The event opens normally and its Overview details are shown — internal staff can view any non-draft event regardless of their own relationship to it.</t>
-        </is>
-      </c>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="14" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="35">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="inlineStr">
+        <is>
+          <t>The event opens normally and its Overview details are shown — internal staff can view any non-draft event regardless of their own relationship to it.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="35">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="35">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="39" t="inlineStr">
-        <is>
-          <t>Kristen</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="35">
       <c r="A15" s="16" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1" s="35">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B16" s="17" t="n">
         <v>46287</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="35"/>
     <row r="17" ht="15.75" customHeight="1" s="35"/>
-    <row r="18" ht="15.75" customHeight="1" s="35">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="35"/>
+    <row r="19" ht="15.75" customHeight="1" s="35">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="35">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="B19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="35">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="39" t="inlineStr">
+      <c r="B20" s="39" t="inlineStr">
         <is>
           <t>The event opens normally and its Overview details are shown with EVT-000209
 Planning</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="35">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="15.75" customHeight="1" s="35">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="35">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B22" s="39" t="inlineStr">
-        <is>
-          <t>Janelle</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="35">
       <c r="A23" s="16" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="35">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B24" s="17" t="n">
         <v>46290</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="35"/>
     <row r="25" ht="15.75" customHeight="1" s="35"/>
     <row r="26" ht="15.75" customHeight="1" s="35"/>
     <row r="27" ht="15.75" customHeight="1" s="35"/>

</xml_diff>